<commit_message>
colores genero y mensaje de error
</commit_message>
<xml_diff>
--- a/data/dict_new.xlsx
+++ b/data/dict_new.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pipei\OneDrive\Escritorio\subn_v3\subnational_gov\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE675BA8-531C-4A65-A935-D18296C6C877}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA0157CC-2C6F-4249-A7B4-D1FAE6635D52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="218">
   <si>
     <t>variable</t>
   </si>
@@ -289,39 +289,21 @@
     <t>date_electoral_sub_leg</t>
   </si>
   <si>
-    <t>Date of the subnational legislative election</t>
-  </si>
-  <si>
     <t>voters_registered_sub_leg</t>
   </si>
   <si>
-    <t>Total registered voters for subnational legislative elections</t>
-  </si>
-  <si>
     <t>total_voters_sub_leg</t>
   </si>
   <si>
-    <t>Total votes cast in subnational legislative elections</t>
-  </si>
-  <si>
     <t>perc_voters_sub_leg</t>
   </si>
   <si>
-    <t>Proportion of registered voters who voted in legislative elections</t>
-  </si>
-  <si>
     <t>valid_votes_sub_leg</t>
   </si>
   <si>
-    <t>Total valid votes in subnational legislative elections</t>
-  </si>
-  <si>
     <t>perc_valid_votes_sub_leg</t>
   </si>
   <si>
-    <t>Percentage of valid votes in legislative elections</t>
-  </si>
-  <si>
     <t>party_name_sub_leg</t>
   </si>
   <si>
@@ -355,30 +337,18 @@
     <t>margin_victory_sub_leg</t>
   </si>
   <si>
-    <t>Difference in vote share between the winner and second-place party (v1 - v2)</t>
-  </si>
-  <si>
     <t>#90A4AE,#00E5FF</t>
   </si>
   <si>
     <t>cumulative_electoral_year_sub_leg</t>
   </si>
   <si>
-    <t>Cumulative count of subnational legislative elections in the state</t>
-  </si>
-  <si>
     <t>concurrent_election_with_nat_sub_leg</t>
   </si>
   <si>
-    <t>Whether subnational legislative and national elections occurred concurrently (1 = Yes, 0 = No)</t>
-  </si>
-  <si>
     <t>num_parties_election_contest_sub_leg</t>
   </si>
   <si>
-    <t>Number of parties contesting subnational legislative elections</t>
-  </si>
-  <si>
     <t>total_seats_in_contest_sub_leg</t>
   </si>
   <si>
@@ -394,21 +364,12 @@
     <t>num_seats_opos_sub_leg</t>
   </si>
   <si>
-    <t>Seats controlled by opposition parties in the subnational legislature</t>
-  </si>
-  <si>
     <t>perc_seats_opos_sub_leg</t>
   </si>
   <si>
-    <t>Percentage of seats controlled by opposition parties</t>
-  </si>
-  <si>
     <t>chamber_sub_leg</t>
   </si>
   <si>
-    <t>Number of chambers in the subnational legislature (1 = Unicameral, 2 = Bicameral)</t>
-  </si>
-  <si>
     <t>#d73027,#4575b4</t>
   </si>
   <si>
@@ -424,9 +385,6 @@
     <t>enp_leg_sub_leg</t>
   </si>
   <si>
-    <t>Effective number of legislative parties in elections (Laakso and Taagepera)</t>
-  </si>
-  <si>
     <t>dataset</t>
   </si>
   <si>
@@ -685,12 +643,6 @@
     <t>Effective number of parties competing in election</t>
   </si>
   <si>
-    <t>Seats controlled by the governor's party in the subnational legislature</t>
-  </si>
-  <si>
-    <t>Percentage of seats controlled by the governor's party</t>
-  </si>
-  <si>
     <t>Voter Turnout Percentage</t>
   </si>
   <si>
@@ -722,6 +674,9 @@
   </si>
   <si>
     <t>Difference in vote percentage between winner and runner-up</t>
+  </si>
+  <si>
+    <t>#C5CA8A,#5E304F,#5FBFF9</t>
   </si>
 </sst>
 </file>
@@ -1069,7 +1024,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:J82"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1098,7 +1052,7 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -1116,7 +1070,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1124,7 +1078,7 @@
         <v>11</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>176</v>
+        <v>162</v>
       </c>
       <c r="D2" t="s">
         <v>10</v>
@@ -1142,7 +1096,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -1150,7 +1104,7 @@
         <v>15</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>177</v>
+        <v>163</v>
       </c>
       <c r="D3" t="s">
         <v>10</v>
@@ -1168,7 +1122,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -1176,7 +1130,7 @@
         <v>19</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>178</v>
+        <v>164</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
@@ -1194,7 +1148,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -1202,7 +1156,7 @@
         <v>22</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="D5" t="s">
         <v>10</v>
@@ -1220,15 +1174,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>180</v>
+        <v>166</v>
       </c>
       <c r="D6" t="s">
         <v>24</v>
@@ -1254,10 +1208,10 @@
         <v>27</v>
       </c>
       <c r="B7" t="s">
-        <v>137</v>
+        <v>123</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>181</v>
+        <v>167</v>
       </c>
       <c r="D7" t="s">
         <v>24</v>
@@ -1281,15 +1235,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>30</v>
       </c>
       <c r="B8" t="s">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>182</v>
+        <v>168</v>
       </c>
       <c r="D8" t="s">
         <v>24</v>
@@ -1310,15 +1264,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>32</v>
       </c>
       <c r="B9" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>183</v>
+        <v>169</v>
       </c>
       <c r="D9" t="s">
         <v>24</v>
@@ -1342,15 +1296,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>34</v>
       </c>
       <c r="B10" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>184</v>
+        <v>170</v>
       </c>
       <c r="D10" t="s">
         <v>24</v>
@@ -1374,15 +1328,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>37</v>
       </c>
       <c r="B11" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>185</v>
+        <v>171</v>
       </c>
       <c r="D11" t="s">
         <v>24</v>
@@ -1406,15 +1360,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>38</v>
       </c>
       <c r="B12" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>186</v>
+        <v>172</v>
       </c>
       <c r="D12" t="s">
         <v>24</v>
@@ -1435,15 +1389,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>143</v>
+        <v>129</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="D13" t="s">
         <v>24</v>
@@ -1467,15 +1421,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="B14" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="D14" t="s">
         <v>24</v>
@@ -1499,15 +1453,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>161</v>
+      </c>
+      <c r="B15" t="s">
+        <v>131</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="B15" t="s">
-        <v>145</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>189</v>
       </c>
       <c r="D15" t="s">
         <v>24</v>
@@ -1533,10 +1487,10 @@
         <v>43</v>
       </c>
       <c r="B16" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>190</v>
+        <v>176</v>
       </c>
       <c r="D16" t="s">
         <v>24</v>
@@ -1548,7 +1502,7 @@
         <v>28</v>
       </c>
       <c r="G16" t="s">
-        <v>29</v>
+        <v>217</v>
       </c>
       <c r="H16">
         <v>1</v>
@@ -1560,15 +1514,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>44</v>
       </c>
       <c r="B17" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>191</v>
+        <v>177</v>
       </c>
       <c r="D17" t="s">
         <v>24</v>
@@ -1589,15 +1543,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>45</v>
       </c>
       <c r="B18" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>192</v>
+        <v>178</v>
       </c>
       <c r="D18" t="s">
         <v>24</v>
@@ -1621,15 +1575,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>46</v>
       </c>
       <c r="B19" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>193</v>
+        <v>179</v>
       </c>
       <c r="D19" t="s">
         <v>24</v>
@@ -1653,15 +1607,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>47</v>
       </c>
       <c r="B20" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>194</v>
+        <v>180</v>
       </c>
       <c r="D20" t="s">
         <v>24</v>
@@ -1685,15 +1639,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>48</v>
       </c>
       <c r="B21" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>195</v>
+        <v>181</v>
       </c>
       <c r="D21" t="s">
         <v>49</v>
@@ -1717,15 +1671,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>51</v>
       </c>
       <c r="B22" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>196</v>
+        <v>182</v>
       </c>
       <c r="D22" t="s">
         <v>49</v>
@@ -1749,15 +1703,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>52</v>
       </c>
       <c r="B23" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>197</v>
+        <v>183</v>
       </c>
       <c r="D23" t="s">
         <v>24</v>
@@ -1781,15 +1735,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>53</v>
       </c>
       <c r="B24" t="s">
-        <v>154</v>
+        <v>140</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="D24" t="s">
         <v>24</v>
@@ -1810,15 +1764,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>54</v>
       </c>
       <c r="B25" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
       <c r="D25" t="s">
         <v>24</v>
@@ -1842,15 +1796,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>55</v>
       </c>
       <c r="B26" t="s">
-        <v>156</v>
+        <v>142</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>200</v>
+        <v>186</v>
       </c>
       <c r="D26" t="s">
         <v>24</v>
@@ -1874,15 +1828,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>56</v>
       </c>
       <c r="B27" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>201</v>
+        <v>187</v>
       </c>
       <c r="D27" t="s">
         <v>24</v>
@@ -1906,15 +1860,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>57</v>
       </c>
       <c r="B28" t="s">
-        <v>158</v>
+        <v>144</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="D28" t="s">
         <v>24</v>
@@ -1938,15 +1892,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>58</v>
       </c>
       <c r="B29" t="s">
-        <v>159</v>
+        <v>145</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="D29" t="s">
         <v>49</v>
@@ -1970,47 +1924,47 @@
         <v>20</v>
       </c>
     </row>
-    <row r="30" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="30" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B30" t="s">
-        <v>160</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="D30" t="s">
-        <v>49</v>
-      </c>
-      <c r="E30" t="s">
+      <c r="B30" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E30" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G30" t="s">
+      <c r="G30" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="H30">
-        <v>1</v>
-      </c>
-      <c r="I30">
-        <v>1</v>
-      </c>
-      <c r="J30" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H30" s="1">
+        <v>1</v>
+      </c>
+      <c r="I30" s="1">
+        <v>1</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>60</v>
       </c>
       <c r="B31" t="s">
-        <v>161</v>
+        <v>147</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>205</v>
+        <v>191</v>
       </c>
       <c r="D31" t="s">
         <v>24</v>
@@ -2034,15 +1988,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>61</v>
       </c>
       <c r="B32" t="s">
-        <v>162</v>
+        <v>148</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>206</v>
+        <v>192</v>
       </c>
       <c r="D32" t="s">
         <v>24</v>
@@ -2066,15 +2020,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>62</v>
       </c>
       <c r="B33" t="s">
-        <v>163</v>
+        <v>149</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>207</v>
+        <v>193</v>
       </c>
       <c r="D33" t="s">
         <v>49</v>
@@ -2098,15 +2052,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="34" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>63</v>
       </c>
       <c r="B34" t="s">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="D34" t="s">
         <v>49</v>
@@ -2127,15 +2081,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>64</v>
       </c>
       <c r="B35" t="s">
-        <v>165</v>
+        <v>151</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="D35" t="s">
         <v>49</v>
@@ -2159,15 +2113,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="36" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>66</v>
       </c>
       <c r="B36" t="s">
-        <v>166</v>
+        <v>152</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="D36" t="s">
         <v>49</v>
@@ -2191,15 +2145,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="37" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>67</v>
       </c>
       <c r="B37" t="s">
-        <v>222</v>
+        <v>206</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>223</v>
+        <v>207</v>
       </c>
       <c r="D37" t="s">
         <v>49</v>
@@ -2223,15 +2177,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="38" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>70</v>
       </c>
       <c r="B38" t="s">
-        <v>167</v>
+        <v>153</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>211</v>
+        <v>197</v>
       </c>
       <c r="D38" t="s">
         <v>49</v>
@@ -2255,15 +2209,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="39" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>71</v>
       </c>
       <c r="B39" t="s">
-        <v>224</v>
+        <v>208</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>212</v>
+        <v>198</v>
       </c>
       <c r="D39" t="s">
         <v>49</v>
@@ -2287,15 +2241,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="40" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>72</v>
       </c>
       <c r="B40" t="s">
-        <v>168</v>
+        <v>154</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>213</v>
+        <v>199</v>
       </c>
       <c r="D40" t="s">
         <v>49</v>
@@ -2319,15 +2273,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="41" spans="1:10" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>73</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>225</v>
+        <v>209</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>214</v>
+        <v>200</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>49</v>
@@ -2351,15 +2305,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="42" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>74</v>
       </c>
       <c r="B42" t="s">
-        <v>169</v>
+        <v>155</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>215</v>
+        <v>201</v>
       </c>
       <c r="D42" t="s">
         <v>49</v>
@@ -2383,15 +2337,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="43" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>75</v>
       </c>
       <c r="B43" t="s">
-        <v>226</v>
+        <v>210</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>227</v>
+        <v>211</v>
       </c>
       <c r="D43" t="s">
         <v>49</v>
@@ -2415,15 +2369,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>76</v>
       </c>
       <c r="B44" t="s">
-        <v>170</v>
+        <v>156</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>216</v>
+        <v>202</v>
       </c>
       <c r="D44" t="s">
         <v>49</v>
@@ -2447,15 +2401,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>77</v>
       </c>
       <c r="B45" t="s">
-        <v>228</v>
+        <v>212</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>229</v>
+        <v>213</v>
       </c>
       <c r="D45" t="s">
         <v>49</v>
@@ -2479,15 +2433,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="46" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>78</v>
       </c>
       <c r="B46" t="s">
-        <v>171</v>
+        <v>157</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>217</v>
+        <v>203</v>
       </c>
       <c r="D46" t="s">
         <v>49</v>
@@ -2511,15 +2465,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>79</v>
       </c>
       <c r="B47" t="s">
-        <v>231</v>
+        <v>215</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>230</v>
+        <v>214</v>
       </c>
       <c r="D47" t="s">
         <v>49</v>
@@ -2543,15 +2497,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="48" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>80</v>
       </c>
       <c r="B48" t="s">
-        <v>172</v>
+        <v>158</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>232</v>
+        <v>216</v>
       </c>
       <c r="D48" t="s">
         <v>49</v>
@@ -2575,15 +2529,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="49" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>81</v>
       </c>
       <c r="B49" t="s">
-        <v>173</v>
+        <v>159</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>218</v>
+        <v>204</v>
       </c>
       <c r="D49" t="s">
         <v>49</v>
@@ -2607,15 +2561,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="50" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>82</v>
       </c>
       <c r="B50" t="s">
-        <v>174</v>
+        <v>160</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>219</v>
+        <v>205</v>
       </c>
       <c r="D50" t="s">
         <v>49</v>
@@ -2639,7 +2593,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="51" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>84</v>
       </c>
@@ -2650,13 +2604,10 @@
         <v>86</v>
       </c>
     </row>
-    <row r="52" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>87</v>
       </c>
-      <c r="C52" s="2" t="s">
-        <v>88</v>
-      </c>
       <c r="D52" t="s">
         <v>49</v>
       </c>
@@ -2673,12 +2624,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="53" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>89</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D53" t="s">
         <v>49</v>
@@ -2696,12 +2644,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="54" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>91</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D54" t="s">
         <v>49</v>
@@ -2719,12 +2664,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="55" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>93</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D55" t="s">
         <v>49</v>
@@ -2745,12 +2687,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="56" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>95</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D56" t="s">
         <v>49</v>
@@ -2768,12 +2707,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="57" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>97</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D57" t="s">
         <v>49</v>
@@ -2794,9 +2730,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="58" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="D58" t="s">
         <v>49</v>
@@ -2805,9 +2741,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="59" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D59" t="s">
         <v>49</v>
@@ -2816,9 +2752,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="60" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D60" t="s">
         <v>49</v>
@@ -2827,9 +2763,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="61" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D61" t="s">
         <v>49</v>
@@ -2838,9 +2774,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="62" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="D62" t="s">
         <v>49</v>
@@ -2849,9 +2785,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="63" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="D63" t="s">
         <v>49</v>
@@ -2860,9 +2796,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="64" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="D64" t="s">
         <v>49</v>
@@ -2871,9 +2807,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="65" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D65" t="s">
         <v>49</v>
@@ -2882,9 +2818,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="66" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="D66" t="s">
         <v>49</v>
@@ -2893,9 +2829,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="67" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="D67" t="s">
         <v>49</v>
@@ -2904,12 +2840,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="68" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>109</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="D68" t="s">
         <v>49</v>
@@ -2927,12 +2860,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="69" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>112</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="D69" t="s">
         <v>49</v>
@@ -2950,12 +2880,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="70" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>114</v>
-      </c>
-      <c r="C70" s="2" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="D70" t="s">
         <v>49</v>
@@ -2964,7 +2891,7 @@
         <v>86</v>
       </c>
       <c r="G70" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="H70">
         <v>0</v>
@@ -2976,12 +2903,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="71" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>116</v>
-      </c>
-      <c r="C71" s="2" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="D71" t="s">
         <v>49</v>
@@ -2999,9 +2923,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="72" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="D72" t="s">
         <v>49</v>
@@ -3010,9 +2934,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="73" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="D73" t="s">
         <v>49</v>
@@ -3021,12 +2945,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="74" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>120</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>220</v>
+        <v>110</v>
       </c>
       <c r="D74" t="s">
         <v>49</v>
@@ -3044,12 +2965,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="75" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>121</v>
-      </c>
-      <c r="C75" s="2" t="s">
-        <v>221</v>
+        <v>111</v>
       </c>
       <c r="D75" t="s">
         <v>49</v>
@@ -3070,12 +2988,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="76" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>122</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="D76" t="s">
         <v>49</v>
@@ -3093,12 +3008,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="77" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>124</v>
-      </c>
-      <c r="C77" s="2" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="D77" t="s">
         <v>49</v>
@@ -3119,12 +3031,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="78" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>126</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="D78" t="s">
         <v>49</v>
@@ -3133,7 +3042,7 @@
         <v>86</v>
       </c>
       <c r="G78" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
       <c r="H78">
         <v>0</v>
@@ -3145,9 +3054,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="79" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="D79" t="s">
         <v>49</v>
@@ -3156,9 +3065,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="80" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="D80" t="s">
         <v>49</v>
@@ -3167,9 +3076,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="81" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="D81" t="s">
         <v>49</v>
@@ -3178,12 +3087,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="82" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>132</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="D82" t="s">
         <v>49</v>
@@ -3202,13 +3108,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J82" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="gender"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:J82" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
screenshot button disable in portrait
</commit_message>
<xml_diff>
--- a/data/dict_new.xlsx
+++ b/data/dict_new.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pipei\OneDrive\Escritorio\subn_v3\subnational_gov\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FC1DF1A-62DB-4BC5-9E6B-5F09EB19BC83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5B48CEC-7BB9-45AA-A835-DE6B91B3D36A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="688" uniqueCount="317">
   <si>
     <t>variable</t>
   </si>
@@ -956,6 +956,24 @@
   </si>
   <si>
     <t>Leg. Elections Concurrent with Nat. Elections</t>
+  </si>
+  <si>
+    <t>add_indices</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Higher values indicate cleaner elections at the subnational executive level, reflecting lower post-electoral conflict.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Higher values indicate higher levels of subnational legistlative competitiveness.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Higher values indicate higher levels of subnational executive competitiveness.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Higher values indicate higher levels of subnational democracy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Higher values indicate higher levels of subnational executive turnover.</t>
   </si>
 </sst>
 </file>
@@ -1330,7 +1348,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:K88"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46.42578125" bestFit="1" customWidth="1"/>
@@ -1344,7 +1362,7 @@
     <col min="9" max="9" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1375,8 +1393,11 @@
       <c r="J1" s="1" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>267</v>
       </c>
@@ -1404,8 +1425,11 @@
       <c r="J2" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>268</v>
       </c>
@@ -1433,8 +1457,11 @@
       <c r="J3" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K3" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>269</v>
       </c>
@@ -1462,8 +1489,11 @@
       <c r="J4" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K4" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>270</v>
       </c>
@@ -1491,8 +1521,11 @@
       <c r="J5" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K5" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>271</v>
       </c>
@@ -1520,8 +1553,11 @@
       <c r="J6" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K6" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>272</v>
       </c>
@@ -1549,8 +1585,11 @@
       <c r="J7" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K7" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1579,7 +1618,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -1608,7 +1647,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1637,7 +1676,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1666,7 +1705,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -1695,7 +1734,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -1727,7 +1766,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1756,7 +1795,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>36</v>
       </c>
@@ -1788,7 +1827,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>39</v>
       </c>

</xml_diff>

<commit_message>
tab duration and cleaning
</commit_message>
<xml_diff>
--- a/data/dict_new.xlsx
+++ b/data/dict_new.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pipei\OneDrive\Escritorio\subn_v3\subnational_gov\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5B48CEC-7BB9-45AA-A835-DE6B91B3D36A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62B761E4-7A32-477A-B922-D4DD6BD1716C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -871,9 +871,6 @@
     <t>#FDE0DD,#FBB4B9,#F768A1,#C51B8A</t>
   </si>
   <si>
-    <t>#F2F2F7,#D9E0EE,#AEB8D0,#7A86A2</t>
-  </si>
-  <si>
     <t>#F4E6F8,#E0C2F0,#C08AE0,#8C4CB8</t>
   </si>
   <si>
@@ -973,7 +970,10 @@
     <t xml:space="preserve"> Higher values indicate higher levels of subnational democracy.</t>
   </si>
   <si>
-    <t xml:space="preserve"> Higher values indicate higher levels of subnational executive turnover.</t>
+    <t>#C0D2EB,#4257A8</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Higher values indicate higher subnational executive turnover.</t>
   </si>
 </sst>
 </file>
@@ -1394,7 +1394,7 @@
         <v>187</v>
       </c>
       <c r="K1" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -1402,7 +1402,7 @@
         <v>267</v>
       </c>
       <c r="B2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D2" t="s">
         <v>276</v>
@@ -1411,7 +1411,7 @@
         <v>121</v>
       </c>
       <c r="F2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -1426,7 +1426,7 @@
         <v>273</v>
       </c>
       <c r="K2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -1443,7 +1443,7 @@
         <v>121</v>
       </c>
       <c r="F3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -1458,7 +1458,7 @@
         <v>274</v>
       </c>
       <c r="K3" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -1466,7 +1466,7 @@
         <v>269</v>
       </c>
       <c r="B4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D4" t="s">
         <v>276</v>
@@ -1475,7 +1475,7 @@
         <v>121</v>
       </c>
       <c r="F4" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -1490,7 +1490,7 @@
         <v>277</v>
       </c>
       <c r="K4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -1498,7 +1498,7 @@
         <v>270</v>
       </c>
       <c r="B5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D5" t="s">
         <v>276</v>
@@ -1507,7 +1507,7 @@
         <v>121</v>
       </c>
       <c r="F5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -1522,7 +1522,7 @@
         <v>278</v>
       </c>
       <c r="K5" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -1530,7 +1530,7 @@
         <v>271</v>
       </c>
       <c r="B6" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D6" t="s">
         <v>276</v>
@@ -1539,7 +1539,7 @@
         <v>121</v>
       </c>
       <c r="F6" t="s">
-        <v>282</v>
+        <v>315</v>
       </c>
       <c r="G6">
         <v>1</v>
@@ -1562,7 +1562,7 @@
         <v>272</v>
       </c>
       <c r="B7" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D7" t="s">
         <v>276</v>
@@ -1586,7 +1586,7 @@
         <v>280</v>
       </c>
       <c r="K7" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -2484,7 +2484,7 @@
         <v>22</v>
       </c>
       <c r="J36" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
@@ -2492,7 +2492,7 @@
         <v>85</v>
       </c>
       <c r="B37" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C37" t="s">
         <v>68</v>
@@ -2524,7 +2524,7 @@
         <v>87</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C38" t="s">
         <v>21</v>
@@ -2556,7 +2556,7 @@
         <v>88</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C39" t="s">
         <v>21</v>
@@ -2713,7 +2713,7 @@
         <v>98</v>
       </c>
       <c r="B44" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C44" t="s">
         <v>68</v>
@@ -2777,7 +2777,7 @@
         <v>103</v>
       </c>
       <c r="B46" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C46" t="s">
         <v>68</v>
@@ -2841,7 +2841,7 @@
         <v>106</v>
       </c>
       <c r="B48" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C48" t="s">
         <v>68</v>
@@ -2905,7 +2905,7 @@
         <v>109</v>
       </c>
       <c r="B50" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C50" t="s">
         <v>68</v>
@@ -2969,7 +2969,7 @@
         <v>112</v>
       </c>
       <c r="B52" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C52" t="s">
         <v>68</v>
@@ -3033,7 +3033,7 @@
         <v>115</v>
       </c>
       <c r="B54" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C54" t="s">
         <v>68</v>
@@ -3065,7 +3065,7 @@
         <v>116</v>
       </c>
       <c r="B55" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C55" t="s">
         <v>68</v>
@@ -3182,7 +3182,7 @@
         <v>22</v>
       </c>
       <c r="J58" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
@@ -3254,7 +3254,7 @@
         <v>130</v>
       </c>
       <c r="B61" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C61" t="s">
         <v>68</v>
@@ -3318,7 +3318,7 @@
         <v>133</v>
       </c>
       <c r="B63" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C63" t="s">
         <v>68</v>
@@ -3507,7 +3507,7 @@
         <v>144</v>
       </c>
       <c r="B69" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C69" t="s">
         <v>68</v>
@@ -3571,7 +3571,7 @@
         <v>147</v>
       </c>
       <c r="B71" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C71" t="s">
         <v>68</v>
@@ -3731,7 +3731,7 @@
         <v>156</v>
       </c>
       <c r="B76" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C76" t="s">
         <v>68</v>
@@ -3795,7 +3795,7 @@
         <v>159</v>
       </c>
       <c r="B78" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C78" t="s">
         <v>68</v>
@@ -3827,7 +3827,7 @@
         <v>160</v>
       </c>
       <c r="B79" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C79" t="s">
         <v>68</v>
@@ -4071,7 +4071,7 @@
         <v>185</v>
       </c>
       <c r="B87" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C87" t="s">
         <v>175</v>
@@ -4100,7 +4100,7 @@
         <v>186</v>
       </c>
       <c r="B88" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C88" t="s">
         <v>175</v>

</xml_diff>

<commit_message>
Revert "Merge branch 'main' into test"
This reverts commit 8e8b7f08365a4aa39a7772ebad2a8df2212b77c9, reversing
changes made to 26fdb06426fe4b53ed7884632c9278316adebb37.
</commit_message>
<xml_diff>
--- a/data/dict_new.xlsx
+++ b/data/dict_new.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pipei\OneDrive\Escritorio\subn_v3\subnational_gov\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62B761E4-7A32-477A-B922-D4DD6BD1716C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FC1DF1A-62DB-4BC5-9E6B-5F09EB19BC83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="688" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="311">
   <si>
     <t>variable</t>
   </si>
@@ -871,6 +871,9 @@
     <t>#FDE0DD,#FBB4B9,#F768A1,#C51B8A</t>
   </si>
   <si>
+    <t>#F2F2F7,#D9E0EE,#AEB8D0,#7A86A2</t>
+  </si>
+  <si>
     <t>#F4E6F8,#E0C2F0,#C08AE0,#8C4CB8</t>
   </si>
   <si>
@@ -953,27 +956,6 @@
   </si>
   <si>
     <t>Leg. Elections Concurrent with Nat. Elections</t>
-  </si>
-  <si>
-    <t>add_indices</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Higher values indicate cleaner elections at the subnational executive level, reflecting lower post-electoral conflict.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Higher values indicate higher levels of subnational legistlative competitiveness.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Higher values indicate higher levels of subnational executive competitiveness.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Higher values indicate higher levels of subnational democracy.</t>
-  </si>
-  <si>
-    <t>#C0D2EB,#4257A8</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Higher values indicate higher subnational executive turnover.</t>
   </si>
 </sst>
 </file>
@@ -1348,7 +1330,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K88"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46.42578125" bestFit="1" customWidth="1"/>
@@ -1362,7 +1344,7 @@
     <col min="9" max="9" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1393,16 +1375,13 @@
       <c r="J1" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="K1" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>267</v>
       </c>
       <c r="B2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D2" t="s">
         <v>276</v>
@@ -1411,7 +1390,7 @@
         <v>121</v>
       </c>
       <c r="F2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -1425,11 +1404,8 @@
       <c r="J2" t="s">
         <v>273</v>
       </c>
-      <c r="K2" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>268</v>
       </c>
@@ -1443,7 +1419,7 @@
         <v>121</v>
       </c>
       <c r="F3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -1457,16 +1433,13 @@
       <c r="J3" t="s">
         <v>274</v>
       </c>
-      <c r="K3" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>269</v>
       </c>
       <c r="B4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D4" t="s">
         <v>276</v>
@@ -1475,7 +1448,7 @@
         <v>121</v>
       </c>
       <c r="F4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -1489,16 +1462,13 @@
       <c r="J4" t="s">
         <v>277</v>
       </c>
-      <c r="K4" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>270</v>
       </c>
       <c r="B5" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D5" t="s">
         <v>276</v>
@@ -1507,7 +1477,7 @@
         <v>121</v>
       </c>
       <c r="F5" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -1521,16 +1491,13 @@
       <c r="J5" t="s">
         <v>278</v>
       </c>
-      <c r="K5" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>271</v>
       </c>
       <c r="B6" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D6" t="s">
         <v>276</v>
@@ -1539,7 +1506,7 @@
         <v>121</v>
       </c>
       <c r="F6" t="s">
-        <v>315</v>
+        <v>282</v>
       </c>
       <c r="G6">
         <v>1</v>
@@ -1553,16 +1520,13 @@
       <c r="J6" t="s">
         <v>279</v>
       </c>
-      <c r="K6" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>272</v>
       </c>
       <c r="B7" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D7" t="s">
         <v>276</v>
@@ -1585,11 +1549,8 @@
       <c r="J7" t="s">
         <v>280</v>
       </c>
-      <c r="K7" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1618,7 +1579,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -1647,7 +1608,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1676,7 +1637,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1705,7 +1666,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -1734,7 +1695,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -1766,7 +1727,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1795,7 +1756,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>36</v>
       </c>
@@ -1827,7 +1788,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>39</v>
       </c>
@@ -2484,7 +2445,7 @@
         <v>22</v>
       </c>
       <c r="J36" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
@@ -2492,7 +2453,7 @@
         <v>85</v>
       </c>
       <c r="B37" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C37" t="s">
         <v>68</v>
@@ -2524,7 +2485,7 @@
         <v>87</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C38" t="s">
         <v>21</v>
@@ -2556,7 +2517,7 @@
         <v>88</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C39" t="s">
         <v>21</v>
@@ -2713,7 +2674,7 @@
         <v>98</v>
       </c>
       <c r="B44" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C44" t="s">
         <v>68</v>
@@ -2777,7 +2738,7 @@
         <v>103</v>
       </c>
       <c r="B46" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C46" t="s">
         <v>68</v>
@@ -2841,7 +2802,7 @@
         <v>106</v>
       </c>
       <c r="B48" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C48" t="s">
         <v>68</v>
@@ -2905,7 +2866,7 @@
         <v>109</v>
       </c>
       <c r="B50" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C50" t="s">
         <v>68</v>
@@ -2969,7 +2930,7 @@
         <v>112</v>
       </c>
       <c r="B52" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C52" t="s">
         <v>68</v>
@@ -3033,7 +2994,7 @@
         <v>115</v>
       </c>
       <c r="B54" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C54" t="s">
         <v>68</v>
@@ -3065,7 +3026,7 @@
         <v>116</v>
       </c>
       <c r="B55" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C55" t="s">
         <v>68</v>
@@ -3182,7 +3143,7 @@
         <v>22</v>
       </c>
       <c r="J58" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
@@ -3254,7 +3215,7 @@
         <v>130</v>
       </c>
       <c r="B61" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C61" t="s">
         <v>68</v>
@@ -3318,7 +3279,7 @@
         <v>133</v>
       </c>
       <c r="B63" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C63" t="s">
         <v>68</v>
@@ -3507,7 +3468,7 @@
         <v>144</v>
       </c>
       <c r="B69" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C69" t="s">
         <v>68</v>
@@ -3571,7 +3532,7 @@
         <v>147</v>
       </c>
       <c r="B71" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C71" t="s">
         <v>68</v>
@@ -3731,7 +3692,7 @@
         <v>156</v>
       </c>
       <c r="B76" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C76" t="s">
         <v>68</v>
@@ -3795,7 +3756,7 @@
         <v>159</v>
       </c>
       <c r="B78" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C78" t="s">
         <v>68</v>
@@ -3827,7 +3788,7 @@
         <v>160</v>
       </c>
       <c r="B79" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C79" t="s">
         <v>68</v>
@@ -4071,7 +4032,7 @@
         <v>185</v>
       </c>
       <c r="B87" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C87" t="s">
         <v>175</v>
@@ -4100,7 +4061,7 @@
         <v>186</v>
       </c>
       <c r="B88" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C88" t="s">
         <v>175</v>

</xml_diff>